<commit_message>
feat: varredura e atualizacao da semana 28 a 03 com dias 02 e 03 de outubro e recuperacao de 56 lojas
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-27).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-27).xlsx
@@ -935,34 +935,34 @@
     <t>214</t>
   </si>
   <si>
-    <t>33</t>
-  </si>
-  <si>
-    <t>R$ 9.451,70</t>
-  </si>
-  <si>
-    <t>101.1</t>
-  </si>
-  <si>
-    <t>66.0</t>
-  </si>
-  <si>
-    <t>7.46</t>
+    <t>28</t>
+  </si>
+  <si>
+    <t>R$ 9.386,45</t>
+  </si>
+  <si>
+    <t>100.5</t>
+  </si>
+  <si>
+    <t>65.9</t>
+  </si>
+  <si>
+    <t>7.40</t>
   </si>
   <si>
     <t>22.9</t>
   </si>
   <si>
-    <t>8.7</t>
-  </si>
-  <si>
-    <t>6.0</t>
+    <t>8.8</t>
+  </si>
+  <si>
+    <t>6.1</t>
   </si>
   <si>
     <t>29.5%</t>
   </si>
   <si>
-    <t>17.8%</t>
+    <t>17.6%</t>
   </si>
   <si>
     <t>1.3%</t>
@@ -971,7 +971,7 @@
     <t>0.4%</t>
   </si>
   <si>
-    <t>3.0%</t>
+    <t>3.1%</t>
   </si>
   <si>
     <t>0.9%</t>
@@ -986,34 +986,34 @@
     <t>2.8%</t>
   </si>
   <si>
-    <t>6.3%</t>
-  </si>
-  <si>
-    <t>2448.0</t>
-  </si>
-  <si>
-    <t>2073.0</t>
-  </si>
-  <si>
-    <t>148.0</t>
+    <t>6.2%</t>
+  </si>
+  <si>
+    <t>2480.0</t>
+  </si>
+  <si>
+    <t>2098.0</t>
+  </si>
+  <si>
+    <t>151.0</t>
   </si>
   <si>
     <t>42.0</t>
   </si>
   <si>
-    <t>356.0</t>
-  </si>
-  <si>
-    <t>103.0</t>
+    <t>370.0</t>
+  </si>
+  <si>
+    <t>105.0</t>
   </si>
   <si>
     <t>15.0</t>
   </si>
   <si>
-    <t>678.0</t>
-  </si>
-  <si>
-    <t>325.0</t>
+    <t>687.0</t>
+  </si>
+  <si>
+    <t>329.0</t>
   </si>
   <si>
     <t>740.0</t>
@@ -6731,7 +6731,7 @@
         <v>19562</v>
       </c>
       <c r="B36" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C36" s="4">
         <v>51</v>
@@ -6761,35 +6761,93 @@
         <v>58</v>
       </c>
       <c r="L36" s="4"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="8"/>
-      <c r="R36" s="8"/>
-      <c r="S36" s="8"/>
-      <c r="T36" s="9"/>
-      <c r="U36" s="9"/>
-      <c r="V36" s="9"/>
-      <c r="W36" s="9"/>
-      <c r="X36" s="9"/>
-      <c r="Y36" s="9"/>
-      <c r="Z36" s="9"/>
-      <c r="AA36" s="9"/>
-      <c r="AB36" s="9"/>
-      <c r="AC36" s="9"/>
-      <c r="AD36" s="6"/>
-      <c r="AE36" s="6"/>
-      <c r="AF36" s="6"/>
-      <c r="AG36" s="6"/>
-      <c r="AH36" s="6"/>
-      <c r="AI36" s="6"/>
-      <c r="AJ36" s="6"/>
-      <c r="AK36" s="6"/>
-      <c r="AL36" s="6"/>
-      <c r="AM36" s="6"/>
-      <c r="AN36" s="9"/>
-      <c r="AO36" s="6"/>
+      <c r="M36" s="5">
+        <v>6850.7200000000003</v>
+      </c>
+      <c r="N36" s="6">
+        <v>89</v>
+      </c>
+      <c r="O36" s="6">
+        <v>79</v>
+      </c>
+      <c r="P36" s="7">
+        <v>4.7196965909090913</v>
+      </c>
+      <c r="Q36" s="8">
+        <v>23.021518987341771</v>
+      </c>
+      <c r="R36" s="8">
+        <v>11.923246052631578</v>
+      </c>
+      <c r="S36" s="8">
+        <v>7</v>
+      </c>
+      <c r="T36" s="9">
+        <v>0.379746835443038</v>
+      </c>
+      <c r="U36" s="9">
+        <v>0.15189873417721519</v>
+      </c>
+      <c r="V36" s="9">
+        <v>0</v>
+      </c>
+      <c r="W36" s="9">
+        <v>0</v>
+      </c>
+      <c r="X36" s="9">
+        <v>0.11392405063291139</v>
+      </c>
+      <c r="Y36" s="9">
+        <v>0.012658227848101266</v>
+      </c>
+      <c r="Z36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="9">
+        <v>0.050632911392405063</v>
+      </c>
+      <c r="AB36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="6">
+        <v>14</v>
+      </c>
+      <c r="AE36" s="6">
+        <v>12</v>
+      </c>
+      <c r="AF36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH36" s="6">
+        <v>9</v>
+      </c>
+      <c r="AI36" s="6">
+        <v>1</v>
+      </c>
+      <c r="AJ36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK36" s="6">
+        <v>4</v>
+      </c>
+      <c r="AL36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO36" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP36" s="4">
         <v>58</v>
       </c>
@@ -7613,7 +7671,7 @@
         <v>19579</v>
       </c>
       <c r="B42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C42" s="4">
         <v>51</v>
@@ -7643,35 +7701,93 @@
         <v>58</v>
       </c>
       <c r="L42" s="4"/>
-      <c r="M42" s="5"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
-      <c r="P42" s="7"/>
-      <c r="Q42" s="8"/>
-      <c r="R42" s="8"/>
-      <c r="S42" s="8"/>
-      <c r="T42" s="9"/>
-      <c r="U42" s="9"/>
-      <c r="V42" s="9"/>
-      <c r="W42" s="9"/>
-      <c r="X42" s="9"/>
-      <c r="Y42" s="9"/>
-      <c r="Z42" s="9"/>
-      <c r="AA42" s="9"/>
-      <c r="AB42" s="9"/>
-      <c r="AC42" s="9"/>
-      <c r="AD42" s="6"/>
-      <c r="AE42" s="6"/>
-      <c r="AF42" s="6"/>
-      <c r="AG42" s="6"/>
-      <c r="AH42" s="6"/>
-      <c r="AI42" s="6"/>
-      <c r="AJ42" s="6"/>
-      <c r="AK42" s="6"/>
-      <c r="AL42" s="6"/>
-      <c r="AM42" s="6"/>
-      <c r="AN42" s="9"/>
-      <c r="AO42" s="6"/>
+      <c r="M42" s="5">
+        <v>7347.4399999999996</v>
+      </c>
+      <c r="N42" s="6">
+        <v>80</v>
+      </c>
+      <c r="O42" s="6">
+        <v>60</v>
+      </c>
+      <c r="P42" s="7">
+        <v>6.0517089743589745</v>
+      </c>
+      <c r="Q42" s="8">
+        <v>22.573611666666668</v>
+      </c>
+      <c r="R42" s="8">
+        <v>9.3375711864406785</v>
+      </c>
+      <c r="S42" s="8">
+        <v>7</v>
+      </c>
+      <c r="T42" s="9">
+        <v>0.083333333333333329</v>
+      </c>
+      <c r="U42" s="9">
+        <v>0.016666666666666666</v>
+      </c>
+      <c r="V42" s="9">
+        <v>0</v>
+      </c>
+      <c r="W42" s="9">
+        <v>0</v>
+      </c>
+      <c r="X42" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="9">
+        <v>0.016666666666666666</v>
+      </c>
+      <c r="AB42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD42" s="6">
+        <v>1</v>
+      </c>
+      <c r="AE42" s="6">
+        <v>1</v>
+      </c>
+      <c r="AF42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK42" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO42" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP42" s="4">
         <v>58</v>
       </c>
@@ -8962,7 +9078,7 @@
         <v>19602</v>
       </c>
       <c r="B51" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C51" s="4">
         <v>51</v>
@@ -8992,35 +9108,93 @@
         <v>58</v>
       </c>
       <c r="L51" s="4"/>
-      <c r="M51" s="5"/>
-      <c r="N51" s="6"/>
-      <c r="O51" s="6"/>
-      <c r="P51" s="7"/>
-      <c r="Q51" s="8"/>
-      <c r="R51" s="8"/>
-      <c r="S51" s="8"/>
-      <c r="T51" s="9"/>
-      <c r="U51" s="9"/>
-      <c r="V51" s="9"/>
-      <c r="W51" s="9"/>
-      <c r="X51" s="9"/>
-      <c r="Y51" s="9"/>
-      <c r="Z51" s="9"/>
-      <c r="AA51" s="9"/>
-      <c r="AB51" s="9"/>
-      <c r="AC51" s="9"/>
-      <c r="AD51" s="6"/>
-      <c r="AE51" s="6"/>
-      <c r="AF51" s="6"/>
-      <c r="AG51" s="6"/>
-      <c r="AH51" s="6"/>
-      <c r="AI51" s="6"/>
-      <c r="AJ51" s="6"/>
-      <c r="AK51" s="6"/>
-      <c r="AL51" s="6"/>
-      <c r="AM51" s="6"/>
-      <c r="AN51" s="9"/>
-      <c r="AO51" s="6"/>
+      <c r="M51" s="5">
+        <v>1213.48</v>
+      </c>
+      <c r="N51" s="6">
+        <v>11</v>
+      </c>
+      <c r="O51" s="6">
+        <v>8</v>
+      </c>
+      <c r="P51" s="7">
+        <v>1.8500000000000001</v>
+      </c>
+      <c r="Q51" s="8">
+        <v>8.7145875000000004</v>
+      </c>
+      <c r="R51" s="8">
+        <v>1.0805499999999999</v>
+      </c>
+      <c r="S51" s="8">
+        <v>7</v>
+      </c>
+      <c r="T51" s="9">
+        <v>1</v>
+      </c>
+      <c r="U51" s="9">
+        <v>0.875</v>
+      </c>
+      <c r="V51" s="9">
+        <v>0</v>
+      </c>
+      <c r="W51" s="9">
+        <v>0</v>
+      </c>
+      <c r="X51" s="9">
+        <v>0.375</v>
+      </c>
+      <c r="Y51" s="9">
+        <v>0.125</v>
+      </c>
+      <c r="Z51" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA51" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AB51" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="AC51" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD51" s="6">
+        <v>12</v>
+      </c>
+      <c r="AE51" s="6">
+        <v>7</v>
+      </c>
+      <c r="AF51" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG51" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH51" s="6">
+        <v>3</v>
+      </c>
+      <c r="AI51" s="6">
+        <v>1</v>
+      </c>
+      <c r="AJ51" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK51" s="6">
+        <v>4</v>
+      </c>
+      <c r="AL51" s="6">
+        <v>4</v>
+      </c>
+      <c r="AM51" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN51" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO51" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP51" s="4">
         <v>58</v>
       </c>
@@ -10031,33 +10205,79 @@
       <c r="L58" s="4"/>
       <c r="M58" s="5"/>
       <c r="N58" s="6"/>
-      <c r="O58" s="6"/>
+      <c r="O58" s="6">
+        <v>100</v>
+      </c>
       <c r="P58" s="7"/>
       <c r="Q58" s="8"/>
       <c r="R58" s="8"/>
-      <c r="S58" s="8"/>
+      <c r="S58" s="8">
+        <v>7</v>
+      </c>
       <c r="T58" s="9"/>
-      <c r="U58" s="9"/>
-      <c r="V58" s="9"/>
-      <c r="W58" s="9"/>
-      <c r="X58" s="9"/>
-      <c r="Y58" s="9"/>
-      <c r="Z58" s="9"/>
-      <c r="AA58" s="9"/>
-      <c r="AB58" s="9"/>
-      <c r="AC58" s="9"/>
-      <c r="AD58" s="6"/>
-      <c r="AE58" s="6"/>
-      <c r="AF58" s="6"/>
-      <c r="AG58" s="6"/>
-      <c r="AH58" s="6"/>
-      <c r="AI58" s="6"/>
-      <c r="AJ58" s="6"/>
-      <c r="AK58" s="6"/>
-      <c r="AL58" s="6"/>
-      <c r="AM58" s="6"/>
-      <c r="AN58" s="9"/>
-      <c r="AO58" s="6"/>
+      <c r="U58" s="9">
+        <v>0.050000000000000003</v>
+      </c>
+      <c r="V58" s="9">
+        <v>0.029999999999999999</v>
+      </c>
+      <c r="W58" s="9">
+        <v>0</v>
+      </c>
+      <c r="X58" s="9">
+        <v>0.02</v>
+      </c>
+      <c r="Y58" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z58" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA58" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB58" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC58" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD58" s="6">
+        <v>5</v>
+      </c>
+      <c r="AE58" s="6">
+        <v>5</v>
+      </c>
+      <c r="AF58" s="6">
+        <v>3</v>
+      </c>
+      <c r="AG58" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH58" s="6">
+        <v>2</v>
+      </c>
+      <c r="AI58" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ58" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK58" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL58" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM58" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN58" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO58" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP58" s="4">
         <v>58</v>
       </c>
@@ -16411,7 +16631,7 @@
         <v>19719</v>
       </c>
       <c r="B102" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C102" s="4">
         <v>51</v>
@@ -16441,14 +16661,26 @@
         <v>58</v>
       </c>
       <c r="L102" s="4"/>
-      <c r="M102" s="5"/>
-      <c r="N102" s="6"/>
+      <c r="M102" s="5">
+        <v>8059.6300000000001</v>
+      </c>
+      <c r="N102" s="6">
+        <v>87</v>
+      </c>
       <c r="O102" s="6"/>
-      <c r="P102" s="7"/>
-      <c r="Q102" s="8"/>
-      <c r="R102" s="8"/>
+      <c r="P102" s="7">
+        <v>9.7945079545454536</v>
+      </c>
+      <c r="Q102" s="8">
+        <v>38.990303636363635</v>
+      </c>
+      <c r="R102" s="8">
+        <v>41.501307843137255</v>
+      </c>
       <c r="S102" s="8"/>
-      <c r="T102" s="9"/>
+      <c r="T102" s="9">
+        <v>0.18181818181818182</v>
+      </c>
       <c r="U102" s="9"/>
       <c r="V102" s="9"/>
       <c r="W102" s="9"/>
@@ -30220,7 +30452,7 @@
         <v>19944</v>
       </c>
       <c r="B195" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C195" s="4">
         <v>51</v>
@@ -30250,14 +30482,26 @@
         <v>58</v>
       </c>
       <c r="L195" s="4"/>
-      <c r="M195" s="5"/>
-      <c r="N195" s="6"/>
+      <c r="M195" s="5">
+        <v>11911.48</v>
+      </c>
+      <c r="N195" s="6">
+        <v>131</v>
+      </c>
       <c r="O195" s="6"/>
-      <c r="P195" s="7"/>
-      <c r="Q195" s="8"/>
-      <c r="R195" s="8"/>
+      <c r="P195" s="7">
+        <v>4.5380574803149605</v>
+      </c>
+      <c r="Q195" s="8">
+        <v>19.452355434782611</v>
+      </c>
+      <c r="R195" s="8">
+        <v>8.096519780219781</v>
+      </c>
       <c r="S195" s="8"/>
-      <c r="T195" s="9"/>
+      <c r="T195" s="9">
+        <v>0.19565217391304349</v>
+      </c>
       <c r="U195" s="9"/>
       <c r="V195" s="9"/>
       <c r="W195" s="9"/>

</xml_diff>

<commit_message>
feat: varredura de subida tardia com 43 lojas e 3897 pedidos resgatados e fechamento de 11/10
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-27).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-09-27).xlsx
@@ -935,16 +935,16 @@
     <t>214</t>
   </si>
   <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>R$ 9.386,45</t>
-  </si>
-  <si>
-    <t>100.5</t>
-  </si>
-  <si>
-    <t>65.9</t>
+    <t>26</t>
+  </si>
+  <si>
+    <t>R$ 9.412,17</t>
+  </si>
+  <si>
+    <t>100.6</t>
+  </si>
+  <si>
+    <t>66.3</t>
   </si>
   <si>
     <t>7.40</t>
@@ -956,22 +956,22 @@
     <t>8.8</t>
   </si>
   <si>
-    <t>6.1</t>
-  </si>
-  <si>
-    <t>29.5%</t>
-  </si>
-  <si>
-    <t>17.6%</t>
-  </si>
-  <si>
-    <t>1.3%</t>
+    <t>6.2</t>
+  </si>
+  <si>
+    <t>29.2%</t>
+  </si>
+  <si>
+    <t>17.4%</t>
+  </si>
+  <si>
+    <t>1.2%</t>
   </si>
   <si>
     <t>0.4%</t>
   </si>
   <si>
-    <t>3.1%</t>
+    <t>3.0%</t>
   </si>
   <si>
     <t>0.9%</t>
@@ -983,22 +983,22 @@
     <t>5.8%</t>
   </si>
   <si>
-    <t>2.8%</t>
+    <t>2.7%</t>
   </si>
   <si>
     <t>6.2%</t>
   </si>
   <si>
-    <t>2480.0</t>
-  </si>
-  <si>
-    <t>2098.0</t>
-  </si>
-  <si>
-    <t>151.0</t>
-  </si>
-  <si>
-    <t>42.0</t>
+    <t>2519.0</t>
+  </si>
+  <si>
+    <t>2135.0</t>
+  </si>
+  <si>
+    <t>152.0</t>
+  </si>
+  <si>
+    <t>43.0</t>
   </si>
   <si>
     <t>370.0</t>
@@ -1007,16 +1007,16 @@
     <t>105.0</t>
   </si>
   <si>
-    <t>15.0</t>
-  </si>
-  <si>
-    <t>687.0</t>
-  </si>
-  <si>
-    <t>329.0</t>
-  </si>
-  <si>
-    <t>740.0</t>
+    <t>16.0</t>
+  </si>
+  <si>
+    <t>705.0</t>
+  </si>
+  <si>
+    <t>334.0</t>
+  </si>
+  <si>
+    <t>754.0</t>
   </si>
   <si>
     <t>0.7%</t>
@@ -2209,7 +2209,7 @@
         <v>19507</v>
       </c>
       <c r="B6" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C6" s="4">
         <v>51</v>
@@ -2239,35 +2239,93 @@
         <v>58</v>
       </c>
       <c r="L6" s="4"/>
-      <c r="M6" s="5"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="8"/>
-      <c r="R6" s="8"/>
-      <c r="S6" s="8"/>
-      <c r="T6" s="9"/>
-      <c r="U6" s="9"/>
-      <c r="V6" s="9"/>
-      <c r="W6" s="9"/>
-      <c r="X6" s="9"/>
-      <c r="Y6" s="9"/>
-      <c r="Z6" s="9"/>
-      <c r="AA6" s="9"/>
-      <c r="AB6" s="9"/>
-      <c r="AC6" s="9"/>
-      <c r="AD6" s="6"/>
-      <c r="AE6" s="6"/>
-      <c r="AF6" s="6"/>
-      <c r="AG6" s="6"/>
-      <c r="AH6" s="6"/>
-      <c r="AI6" s="6"/>
-      <c r="AJ6" s="6"/>
-      <c r="AK6" s="6"/>
-      <c r="AL6" s="6"/>
-      <c r="AM6" s="6"/>
-      <c r="AN6" s="9"/>
-      <c r="AO6" s="6"/>
+      <c r="M6" s="5">
+        <v>17227.669999999998</v>
+      </c>
+      <c r="N6" s="6">
+        <v>167</v>
+      </c>
+      <c r="O6" s="6">
+        <v>128</v>
+      </c>
+      <c r="P6" s="7">
+        <v>7.2276769696969705</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>17.619921874999999</v>
+      </c>
+      <c r="R6" s="8">
+        <v>3.4194663999999997</v>
+      </c>
+      <c r="S6" s="8">
+        <v>7</v>
+      </c>
+      <c r="T6" s="9">
+        <v>0.390625</v>
+      </c>
+      <c r="U6" s="9">
+        <v>0.0625</v>
+      </c>
+      <c r="V6" s="9">
+        <v>0</v>
+      </c>
+      <c r="W6" s="9">
+        <v>0</v>
+      </c>
+      <c r="X6" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="9">
+        <v>0.0078125</v>
+      </c>
+      <c r="AA6" s="9">
+        <v>0.0390625</v>
+      </c>
+      <c r="AB6" s="9">
+        <v>0.03125</v>
+      </c>
+      <c r="AC6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD6" s="6">
+        <v>10</v>
+      </c>
+      <c r="AE6" s="6">
+        <v>8</v>
+      </c>
+      <c r="AF6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="6">
+        <v>1</v>
+      </c>
+      <c r="AK6" s="6">
+        <v>5</v>
+      </c>
+      <c r="AL6" s="6">
+        <v>4</v>
+      </c>
+      <c r="AM6" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN6" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO6" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP6" s="4">
         <v>58</v>
       </c>
@@ -7092,7 +7150,7 @@
         <v>11.300000000000001</v>
       </c>
       <c r="S38" s="8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T38" s="9">
         <v>0.14736842105263157</v>
@@ -16667,7 +16725,9 @@
       <c r="N102" s="6">
         <v>87</v>
       </c>
-      <c r="O102" s="6"/>
+      <c r="O102" s="6">
+        <v>62</v>
+      </c>
       <c r="P102" s="7">
         <v>9.7945079545454536</v>
       </c>
@@ -16677,31 +16737,75 @@
       <c r="R102" s="8">
         <v>41.501307843137255</v>
       </c>
-      <c r="S102" s="8"/>
+      <c r="S102" s="8">
+        <v>7</v>
+      </c>
       <c r="T102" s="9">
         <v>0.18181818181818182</v>
       </c>
-      <c r="U102" s="9"/>
-      <c r="V102" s="9"/>
-      <c r="W102" s="9"/>
-      <c r="X102" s="9"/>
-      <c r="Y102" s="9"/>
-      <c r="Z102" s="9"/>
-      <c r="AA102" s="9"/>
-      <c r="AB102" s="9"/>
-      <c r="AC102" s="9"/>
-      <c r="AD102" s="6"/>
-      <c r="AE102" s="6"/>
-      <c r="AF102" s="6"/>
-      <c r="AG102" s="6"/>
-      <c r="AH102" s="6"/>
-      <c r="AI102" s="6"/>
-      <c r="AJ102" s="6"/>
-      <c r="AK102" s="6"/>
-      <c r="AL102" s="6"/>
-      <c r="AM102" s="6"/>
-      <c r="AN102" s="9"/>
-      <c r="AO102" s="6"/>
+      <c r="U102" s="9">
+        <v>0.43548387096774194</v>
+      </c>
+      <c r="V102" s="9">
+        <v>0</v>
+      </c>
+      <c r="W102" s="9">
+        <v>0</v>
+      </c>
+      <c r="X102" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y102" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z102" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA102" s="9">
+        <v>0.19354838709677419</v>
+      </c>
+      <c r="AB102" s="9">
+        <v>0.016129032258064516</v>
+      </c>
+      <c r="AC102" s="9">
+        <v>0.22580645161290322</v>
+      </c>
+      <c r="AD102" s="6">
+        <v>27</v>
+      </c>
+      <c r="AE102" s="6">
+        <v>27</v>
+      </c>
+      <c r="AF102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK102" s="6">
+        <v>12</v>
+      </c>
+      <c r="AL102" s="6">
+        <v>1</v>
+      </c>
+      <c r="AM102" s="6">
+        <v>14</v>
+      </c>
+      <c r="AN102" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO102" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP102" s="4">
         <v>58</v>
       </c>
@@ -24885,7 +24989,7 @@
         <v>19859</v>
       </c>
       <c r="B158" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C158" s="4">
         <v>51</v>
@@ -24915,35 +25019,93 @@
         <v>58</v>
       </c>
       <c r="L158" s="4"/>
-      <c r="M158" s="5"/>
-      <c r="N158" s="6"/>
-      <c r="O158" s="6"/>
-      <c r="P158" s="7"/>
-      <c r="Q158" s="8"/>
-      <c r="R158" s="8"/>
-      <c r="S158" s="8"/>
-      <c r="T158" s="9"/>
-      <c r="U158" s="9"/>
-      <c r="V158" s="9"/>
-      <c r="W158" s="9"/>
-      <c r="X158" s="9"/>
-      <c r="Y158" s="9"/>
-      <c r="Z158" s="9"/>
-      <c r="AA158" s="9"/>
-      <c r="AB158" s="9"/>
-      <c r="AC158" s="9"/>
-      <c r="AD158" s="6"/>
-      <c r="AE158" s="6"/>
-      <c r="AF158" s="6"/>
-      <c r="AG158" s="6"/>
-      <c r="AH158" s="6"/>
-      <c r="AI158" s="6"/>
-      <c r="AJ158" s="6"/>
-      <c r="AK158" s="6"/>
-      <c r="AL158" s="6"/>
-      <c r="AM158" s="6"/>
-      <c r="AN158" s="9"/>
-      <c r="AO158" s="6"/>
+      <c r="M158" s="5">
+        <v>6278.4499999999998</v>
+      </c>
+      <c r="N158" s="6">
+        <v>55</v>
+      </c>
+      <c r="O158" s="6">
+        <v>50</v>
+      </c>
+      <c r="P158" s="7">
+        <v>7.2002982142857146</v>
+      </c>
+      <c r="Q158" s="8">
+        <v>27.006665999999999</v>
+      </c>
+      <c r="R158" s="8">
+        <v>12.595334000000001</v>
+      </c>
+      <c r="S158" s="8">
+        <v>7</v>
+      </c>
+      <c r="T158" s="9">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="U158" s="9">
+        <v>0</v>
+      </c>
+      <c r="V158" s="9">
+        <v>0</v>
+      </c>
+      <c r="W158" s="9">
+        <v>0</v>
+      </c>
+      <c r="X158" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y158" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM158" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN158" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO158" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP158" s="4">
         <v>58</v>
       </c>
@@ -30488,7 +30650,9 @@
       <c r="N195" s="6">
         <v>131</v>
       </c>
-      <c r="O195" s="6"/>
+      <c r="O195" s="6">
+        <v>92</v>
+      </c>
       <c r="P195" s="7">
         <v>4.5380574803149605</v>
       </c>
@@ -30498,31 +30662,75 @@
       <c r="R195" s="8">
         <v>8.096519780219781</v>
       </c>
-      <c r="S195" s="8"/>
+      <c r="S195" s="8">
+        <v>7</v>
+      </c>
       <c r="T195" s="9">
         <v>0.19565217391304349</v>
       </c>
-      <c r="U195" s="9"/>
-      <c r="V195" s="9"/>
-      <c r="W195" s="9"/>
-      <c r="X195" s="9"/>
-      <c r="Y195" s="9"/>
-      <c r="Z195" s="9"/>
-      <c r="AA195" s="9"/>
-      <c r="AB195" s="9"/>
-      <c r="AC195" s="9"/>
-      <c r="AD195" s="6"/>
-      <c r="AE195" s="6"/>
-      <c r="AF195" s="6"/>
-      <c r="AG195" s="6"/>
-      <c r="AH195" s="6"/>
-      <c r="AI195" s="6"/>
-      <c r="AJ195" s="6"/>
-      <c r="AK195" s="6"/>
-      <c r="AL195" s="6"/>
-      <c r="AM195" s="6"/>
-      <c r="AN195" s="9"/>
-      <c r="AO195" s="6"/>
+      <c r="U195" s="9">
+        <v>0.021739130434782608</v>
+      </c>
+      <c r="V195" s="9">
+        <v>0.010869565217391304</v>
+      </c>
+      <c r="W195" s="9">
+        <v>0.010869565217000001</v>
+      </c>
+      <c r="X195" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y195" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA195" s="9">
+        <v>0.010869565217391304</v>
+      </c>
+      <c r="AB195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD195" s="6">
+        <v>2</v>
+      </c>
+      <c r="AE195" s="6">
+        <v>2</v>
+      </c>
+      <c r="AF195" s="6">
+        <v>1</v>
+      </c>
+      <c r="AG195" s="6">
+        <v>1</v>
+      </c>
+      <c r="AH195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK195" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM195" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN195" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO195" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP195" s="4">
         <v>58</v>
       </c>

</xml_diff>